<commit_message>
change config tool to excelconfigcompiler
</commit_message>
<xml_diff>
--- a/Excel/Level.xlsx
+++ b/Excel/Level.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,59 +471,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1_1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H2" t="n">
-        <v>8</v>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1100</v>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1_2</t>
-        </is>
+      <c r="A3" t="n">
+        <v>101</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
         <v>8</v>
@@ -537,29 +551,27 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1_3</t>
-        </is>
+      <c r="A4" t="n">
+        <v>102</v>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G4" t="n">
         <v>8</v>
@@ -573,29 +585,27 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1300</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1_4</t>
-        </is>
+      <c r="A5" t="n">
+        <v>103</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G5" t="n">
         <v>8</v>
@@ -609,101 +619,95 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1_5</t>
-        </is>
+      <c r="A6" t="n">
+        <v>104</v>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
       <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8</v>
+      </c>
+      <c r="H6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>105</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
         <v>5</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>25</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E7" t="n">
         <v>17</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F7" t="n">
         <v>21</v>
       </c>
-      <c r="G6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H6" t="n">
-        <v>8</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
+      <c r="G7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
         <v>1500</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2_1</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>29</v>
-      </c>
-      <c r="E7" t="n">
-        <v>21</v>
-      </c>
-      <c r="F7" t="n">
-        <v>25</v>
-      </c>
-      <c r="G7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" t="n">
-        <v>8</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>1300</v>
-      </c>
-    </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2_2</t>
-        </is>
+      <c r="A8" t="n">
+        <v>201</v>
       </c>
       <c r="B8" t="n">
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
         <v>8</v>
@@ -717,29 +721,27 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2_3</t>
-        </is>
+      <c r="A9" t="n">
+        <v>202</v>
       </c>
       <c r="B9" t="n">
         <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G9" t="n">
         <v>8</v>
@@ -753,29 +755,27 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1500</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2_4</t>
-        </is>
+      <c r="A10" t="n">
+        <v>203</v>
       </c>
       <c r="B10" t="n">
         <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G10" t="n">
         <v>8</v>
@@ -789,42 +789,74 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1600</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2_5</t>
-        </is>
+      <c r="A11" t="n">
+        <v>204</v>
       </c>
       <c r="B11" t="n">
         <v>2</v>
       </c>
       <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E11" t="n">
+        <v>18</v>
+      </c>
+      <c r="F11" t="n">
+        <v>22</v>
+      </c>
+      <c r="G11" t="n">
+        <v>8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>8</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>205</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
         <v>5</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>25</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>17</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F12" t="n">
         <v>21</v>
       </c>
-      <c r="G11" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" t="n">
-        <v>8</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
+      <c r="G12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
         <v>1700</v>
       </c>
     </row>

</xml_diff>